<commit_message>
Roadmap Excel'inde birebir çeviri ifadeleri düzeltildi
"API yüzeyi", "sarmalayıcı", "köprü", "paketlenmesi" gibi zorlama
çeviriler doğal Türkçe açıklamalarla değiştirildi (JSpecify, API
versiyonlama, Spring AI riski ve MCP starter satırları).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/framework-upgrade-roadmap.xlsx
+++ b/framework-upgrade-roadmap.xlsx
@@ -2752,7 +2752,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>zeus-ai-mcp: MCP server starter (tool kayıt API'si, @McpTool sarmalayıcı)</t>
+          <t>zeus-ai-mcp: MCP server starter (tool kayıt API'si, anotasyonla tool tanımı)</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Servis → MCP tool köprüsü</t>
+          <t>Mevcut servis metotları MCP tool olarak yayınlanır</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Spring Framework 7'nin JSpecify null-safety anotasyonlarının zeus API yüzeylerine uygulanması — tüketici uygulamalara derleme zamanı null uyarıları.</t>
+          <t>Spring Framework 7 ile gelen JSpecify anotasyonlarının (@Nullable/@NonNull) zeus modüllerinin dışa açılan sınıf ve metot imzalarına eklenmesi. Kazanım: tüketici uygulamalar null hatasını çalışma zamanında NPE olarak değil, derleme sırasında IDE/derleyici uyarısı olarak yakalar.</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Spring Framework 7'nin yerleşik API versioning desteğinin zeus konvansiyonu olarak paketlenmesi (header/path stratejisi, springdoc entegrasyonu).</t>
+          <t>Spring Framework 7'nin yerleşik API versioning özelliği için zeus genelinde tek bir standart belirlenmesi (header mi path mi, springdoc entegrasyonu) — her uygulama kendi yöntemini icat etmesin.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>BOM'da spring-ai sürüm pinleme; starter API'sine değil zeus sarmalayıcı API'sine kod yazdırma (izolasyon katmanı)</t>
+          <t>BOM'da spring-ai sürüm pinleme; uygulama kodu Spring AI API'sini doğrudan değil zeus-ai-mcp üzerinden kullanır — Spring AI'da API değişirse yalnız zeus modülü güncellenir</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">

</xml_diff>